<commit_message>
Rebuild videos, subtitles, practice file and upload kit without Read_Me
Both videos are 10:45 with 65 steps; the sheet tabs start at Raw_Data.
Subtitles, chapter times and practice task times follow the new timeline.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ADsxUUq9tw7hB68qavRRLp
</commit_message>
<xml_diff>
--- a/Excel_MIS_Tutorial/practice/Sales_MIS_Practice.xlsx
+++ b/Excel_MIS_Tutorial/practice/Sales_MIS_Practice.xlsx
@@ -872,7 +872,7 @@
     <row r="12" ht="46.5" customHeight="1">
       <c r="B12" s="34" t="inlineStr">
         <is>
-          <t>1:55</t>
+          <t>1:46</t>
         </is>
       </c>
       <c r="C12" s="35" t="inlineStr">
@@ -892,7 +892,7 @@
     <row r="13" ht="46.5" customHeight="1">
       <c r="B13" s="34" t="inlineStr">
         <is>
-          <t>2:42</t>
+          <t>2:33</t>
         </is>
       </c>
       <c r="C13" s="35" t="inlineStr">
@@ -912,7 +912,7 @@
     <row r="14" ht="108.5" customHeight="1">
       <c r="B14" s="34" t="inlineStr">
         <is>
-          <t>3:36</t>
+          <t>3:27</t>
         </is>
       </c>
       <c r="C14" s="35" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="15" ht="62" customHeight="1">
       <c r="B15" s="34" t="inlineStr">
         <is>
-          <t>5:17</t>
+          <t>5:08</t>
         </is>
       </c>
       <c r="C15" s="35" t="inlineStr">
@@ -952,7 +952,7 @@
     <row r="16" ht="62" customHeight="1">
       <c r="B16" s="34" t="inlineStr">
         <is>
-          <t>6:19</t>
+          <t>6:10</t>
         </is>
       </c>
       <c r="C16" s="35" t="inlineStr">
@@ -972,7 +972,7 @@
     <row r="17" ht="31" customHeight="1">
       <c r="B17" s="34" t="inlineStr">
         <is>
-          <t>7:24</t>
+          <t>7:15</t>
         </is>
       </c>
       <c r="C17" s="35" t="inlineStr">
@@ -992,7 +992,7 @@
     <row r="18" ht="46.5" customHeight="1">
       <c r="B18" s="34" t="inlineStr">
         <is>
-          <t>8:02</t>
+          <t>7:53</t>
         </is>
       </c>
       <c r="C18" s="35" t="inlineStr">
@@ -1012,7 +1012,7 @@
     <row r="19" ht="31" customHeight="1">
       <c r="B19" s="34" t="inlineStr">
         <is>
-          <t>9:24</t>
+          <t>9:16</t>
         </is>
       </c>
       <c r="C19" s="35" t="inlineStr">

</xml_diff>